<commit_message>
Update example and README subtitle to 500 compounds
</commit_message>
<xml_diff>
--- a/example/xt01_example_output.xlsx
+++ b/example/xt01_example_output.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="xt01(1).txt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'xt01(1).txt'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'xt01(1).txt'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -513,20 +513,20 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9.170500000000001</v>
+        <v>3.1029</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>(E)-2-Hexenal</t>
+          <t>Isoamyl acetate</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>6728-26-3</t>
+          <t>123-92-2</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>906</v>
+        <v>869</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5174</v>
+        <v>712</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>15727644</v>
+        <v>19081374</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>C6H10O</t>
+          <t>C7H14O2</t>
         </is>
       </c>
     </row>
@@ -550,20 +550,20 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>9.4528</v>
+        <v>5.3102</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2-Pentylfuran</t>
+          <t>(Z)-3-Hexenyl propanoate</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>3777-69-3</t>
+          <t>33467-74-2</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -571,14 +571,14 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>209783</v>
+        <v>162659</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>16836329</v>
+        <v>278853916</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>C9H14O</t>
+          <t>C9H16O2</t>
         </is>
       </c>
     </row>
@@ -587,20 +587,20 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>9.690799999999999</v>
+        <v>6.2795</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2-Pentylfuran</t>
+          <t>2-Methylpropyl 2-methylpropanoate</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>3777-69-3</t>
+          <t>97-85-8</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>880</v>
+        <v>872</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -608,14 +608,14 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>38971</v>
+        <v>38285</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>15548939</v>
+        <v>26621410</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>C9H14O</t>
+          <t>C8H16O2</t>
         </is>
       </c>
     </row>
@@ -624,20 +624,20 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>14.8775</v>
+        <v>6.3815</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2,4,6-Trimethylpyridine</t>
+          <t>2-Methylpropyl 2-methylpropanoate</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>108-75-8</t>
+          <t>97-85-8</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -645,14 +645,14 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>9371121</v>
+        <v>16346</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>97785242</v>
+        <v>25427852</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>C8H11N</t>
+          <t>C8H16O2</t>
         </is>
       </c>
     </row>
@@ -661,20 +661,20 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>15.6462</v>
+        <v>8.197699999999999</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Nonanal</t>
+          <t>2-Methylbutyl acetate</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>124-19-6</t>
+          <t>624-41-9</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -682,14 +682,14 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1683168</v>
+        <v>163506</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>25032769</v>
+        <v>17695492</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>C9H18O</t>
+          <t>C7H14O2</t>
         </is>
       </c>
     </row>
@@ -698,20 +698,20 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>18.163</v>
+        <v>9.170500000000001</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1-Penten-3-ol</t>
+          <t>(E)-2-Hexenal</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>616-25-1</t>
+          <t>6728-26-3</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>876</v>
+        <v>906</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -719,14 +719,14 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>915781</v>
+        <v>5174</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>23316526</v>
+        <v>15727644</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>C5H10O</t>
+          <t>C6H10O</t>
         </is>
       </c>
     </row>
@@ -735,20 +735,20 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>19.6221</v>
+        <v>9.4528</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1-Penten-3-ol</t>
+          <t>2-Pentylfuran</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>616-25-1</t>
+          <t>3777-69-3</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -756,14 +756,14 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>473670</v>
+        <v>209783</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>16947374</v>
+        <v>16836329</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>C5H10O</t>
+          <t>C9H14O</t>
         </is>
       </c>
     </row>
@@ -772,20 +772,20 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>20.7887</v>
+        <v>9.690799999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1-Octen-3-one</t>
+          <t>2-Pentylfuran</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>4312-99-6</t>
+          <t>3777-69-3</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>854</v>
+        <v>880</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -793,14 +793,14 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1023167</v>
+        <v>38971</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>24534517</v>
+        <v>15548939</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>C8H14O</t>
+          <t>C9H14O</t>
         </is>
       </c>
     </row>
@@ -809,20 +809,20 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>22.0335</v>
+        <v>13.1124</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1-Octen-3-one</t>
+          <t>2-Methylpropyl 2-methylpropanoate</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>4312-99-6</t>
+          <t>97-85-8</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>872</v>
+        <v>863</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -830,14 +830,14 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>283638</v>
+        <v>1133602</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>14798843</v>
+        <v>19857368</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>C8H14O</t>
+          <t>C8H16O2</t>
         </is>
       </c>
     </row>
@@ -846,20 +846,20 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>23.9687</v>
+        <v>14.8775</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2-Octen-1-ol</t>
+          <t>2,4,6-Trimethylpyridine</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>22104-78-5</t>
+          <t>108-75-8</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>867</v>
+        <v>894</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -867,14 +867,14 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>212489</v>
+        <v>9371121</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>14804588</v>
+        <v>97785242</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>C8H16O</t>
+          <t>C8H11N</t>
         </is>
       </c>
     </row>
@@ -883,20 +883,20 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>27.1862</v>
+        <v>15.6462</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2-Octen-1-ol</t>
+          <t>Nonanal</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>22104-78-5</t>
+          <t>124-19-6</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -904,14 +904,14 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>2090270</v>
+        <v>1683168</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>43612867</v>
+        <v>25032769</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>C8H16O</t>
+          <t>C9H18O</t>
         </is>
       </c>
     </row>
@@ -920,20 +920,20 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>28.4004</v>
+        <v>18.163</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2,4-Hexadienal</t>
+          <t>(Z)-3-Hexenyl propanoate</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>142-83-6</t>
+          <t>33467-74-2</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -941,14 +941,14 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>257611</v>
+        <v>915781</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>14783769</v>
+        <v>23316526</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>C6H8O</t>
+          <t>C9H16O2</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>29.0126</v>
+        <v>19.6221</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -978,10 +978,10 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>559883</v>
+        <v>473670</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>20514461</v>
+        <v>16947374</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -994,20 +994,20 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>29.7302</v>
+        <v>20.7887</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2,4-Hexadienal</t>
+          <t>1-Octen-3-one</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>142-83-6</t>
+          <t>4312-99-6</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>870</v>
+        <v>854</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1015,14 +1015,14 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>634433</v>
+        <v>1023167</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>20742863</v>
+        <v>24534517</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>C6H8O</t>
+          <t>C8H14O</t>
         </is>
       </c>
     </row>
@@ -1031,20 +1031,20 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.2674</v>
+        <v>22.0335</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>beta-Ionone</t>
+          <t>1-Octen-3-one</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>79-77-6</t>
+          <t>4312-99-6</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>897</v>
+        <v>872</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1052,14 +1052,14 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>1073571</v>
+        <v>283638</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>28797968</v>
+        <v>14798843</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>C13H20O</t>
+          <t>C8H14O</t>
         </is>
       </c>
     </row>
@@ -1068,40 +1068,706 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="n">
+        <v>23.9687</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>(Z)-3-Hexenyl propanoate</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>33467-74-2</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>893</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>212489</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>14804588</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>C9H16O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>27.1862</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2-Octen-1-ol</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>22104-78-5</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>888</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>2090270</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>43612867</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>28.4004</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2-Butylfuran</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>4466-24-4</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>883</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>257611</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>14783769</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>C8H12O</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>29.0126</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>1-Penten-3-ol</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>616-25-1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>871</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>559883</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>20514461</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>C5H10O</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>29.5431</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hexyl propanoate</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2445-76-3</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>879</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1156069</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>29363240</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>C9H18O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>29.7302</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2-Butylfuran</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>4466-24-4</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>882</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>634433</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>20742863</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>C8H12O</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>29.9547</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>3,5-Octadien-2-one</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>38284-27-4</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>868</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>945950</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>25976200</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>C8H12O</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>31.6246</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Propyl butanoate</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>105-66-8</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>873</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>846827</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>22638306</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>C7H14O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>31.8661</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Propyl butanoate</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>105-66-8</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>560467</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>17994111</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>C7H14O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>32.0702</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>3,5-Octadien-2-one</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>38284-27-4</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>851</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>484152</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>19041254</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>C8H12O</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>33.2674</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>beta-Ionone</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>79-77-6</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>897</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1073571</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>28797968</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>C13H20O</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="n">
         <v>36.2944</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Hexanoic acid</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>142-62-1</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E28" s="2" t="n">
         <v>904</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>316552</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>17533079</v>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>C6H12O2</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>40.0288</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Methyl 3-methylbutanoate</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>556-24-1</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>852</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>123924</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>15933831</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>C6H12O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>41.5321</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>852</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>7197</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>16462780</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>42.0286</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>866</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>22755</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>19561305</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>42.6136</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>858</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>62914</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>23318349</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>42.8211</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>859</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>48423</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>24267495</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>43.3041</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>855</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>5899</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>26297916</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>44.8108</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Isoamyl lactate</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>19329-89-6</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>856</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>29666</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>28245293</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>C8H16O3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:I35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>